<commit_message>
Add CVF-AE paper completion figures
</commit_message>
<xml_diff>
--- a/routes/route_b_cvf_ae/results/cvf_ae_paper_results_package_20260624_from_formal_results/CVF_AE_PAPER_RESULTS_PACKAGE.xlsx
+++ b/routes/route_b_cvf_ae/results/cvf_ae_paper_results_package_20260624_from_formal_results/CVF_AE_PAPER_RESULTS_PACKAGE.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R843041b4d6054889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Compact" sheetId="2" r:id="Rfb000aa5f6684795"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Long" sheetId="3" r:id="R4f889e31893c4084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Significance" sheetId="4" r:id="R184ebe5c19d844e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablation" sheetId="5" r:id="R547da5a2a55e4afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablation Sig" sheetId="6" r:id="R0990901f86aa4394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="7" r:id="R90e115a5db75403a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overhead" sheetId="8" r:id="R5fa7fd9df60e4acd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="9" r:id="R44bc94e349a54c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure Index" sheetId="10" r:id="R3be0988dda0c40e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4881aa6a29dc4afb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Compact" sheetId="2" r:id="R85d6548b381049f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Long" sheetId="3" r:id="R2927547773f6492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Significance" sheetId="4" r:id="R7c51ae55261c4639"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablation" sheetId="5" r:id="Ra96db164ebe94785"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablation Sig" sheetId="6" r:id="R63f3d778d839466d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="7" r:id="R310f592c1ee04274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overhead" sheetId="8" r:id="R0eb31390b12549bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="9" r:id="R3db9fdf456e44068"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure Index" sheetId="10" r:id="R5df5d6ac55f44b49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -65,7 +65,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -100,6 +100,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -174,7 +204,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="99">
+  <x:cellXfs count="121">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -428,6 +458,72 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -603,14 +699,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="FigureIndexTable" displayName="FigureIndexTable" ref="A1:I22" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="FigureIndexTable" displayName="FigureIndexTable" ref="A1:I26" headerRowCount="1">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="FigureId"/>
     <x:tableColumn id="2" name="Group"/>
     <x:tableColumn id="3" name="Scene"/>
     <x:tableColumn id="4" name="View"/>
     <x:tableColumn id="5" name="FileName"/>
-    <x:tableColumn id="6" name="Placement"/>
+    <x:tableColumn id="6" name="SuggestedPlacement"/>
     <x:tableColumn id="7" name="Purpose"/>
     <x:tableColumn id="8" name="Status"/>
     <x:tableColumn id="9" name="RelativePath"/>
@@ -1023,78 +1119,78 @@
     <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="45" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="13" t="str">
+    <x:row r="1" ht="30" hidden="0" customHeight="1">
+      <x:c r="A1" s="114" t="str">
         <x:v>FigureId</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B1" s="114" t="str">
         <x:v>Group</x:v>
       </x:c>
-      <x:c r="C1" s="13" t="str">
+      <x:c r="C1" s="114" t="str">
         <x:v>Scene</x:v>
       </x:c>
-      <x:c r="D1" s="13" t="str">
+      <x:c r="D1" s="114" t="str">
         <x:v>View</x:v>
       </x:c>
-      <x:c r="E1" s="13" t="str">
+      <x:c r="E1" s="114" t="str">
         <x:v>FileName</x:v>
       </x:c>
-      <x:c r="F1" s="13" t="str">
-        <x:v>Placement</x:v>
-      </x:c>
-      <x:c r="G1" s="13" t="str">
+      <x:c r="F1" s="114" t="str">
+        <x:v>SuggestedPlacement</x:v>
+      </x:c>
+      <x:c r="G1" s="114" t="str">
         <x:v>Purpose</x:v>
       </x:c>
-      <x:c r="H1" s="13" t="str">
+      <x:c r="H1" s="114" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I1" s="13" t="str">
+      <x:c r="I1" s="114" t="str">
         <x:v>RelativePath</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="42" hidden="0" customHeight="1">
-      <x:c r="A2" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="str">
+      <x:c r="A2" s="115" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="115" t="str">
         <x:v>ablation-path</x:v>
       </x:c>
-      <x:c r="C2" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" s="8" t="str">
+      <x:c r="C2" s="115" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="115" t="str">
         <x:v>3d</x:v>
       </x:c>
-      <x:c r="E2" s="14" t="str">
+      <x:c r="E2" s="116" t="str">
         <x:v>ablation_scene1_representative_3d.png</x:v>
       </x:c>
-      <x:c r="F2" s="8" t="str">
+      <x:c r="F2" s="116" t="str">
         <x:v>supplement</x:v>
       </x:c>
-      <x:c r="G2" s="14" t="str">
+      <x:c r="G2" s="116" t="str">
         <x:v>Visualize module contribution and failure cases</x:v>
       </x:c>
-      <x:c r="H2" s="8" t="str">
+      <x:c r="H2" s="116" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I2" s="14" t="str">
+      <x:c r="I2" s="116" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\ablation\ablation_scene1_representative_3d.png</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
-      <x:c r="A3" s="17" t="n">
+      <x:c r="A3" s="8" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
         <x:v>ablation-path</x:v>
       </x:c>
-      <x:c r="C3" s="17" t="n">
+      <x:c r="C3" s="8" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
@@ -1103,13 +1199,13 @@
       <x:c r="E3" s="14" t="str">
         <x:v>ablation_scene1_representative_top.png</x:v>
       </x:c>
-      <x:c r="F3" s="8" t="str">
+      <x:c r="F3" s="14" t="str">
         <x:v>supplement</x:v>
       </x:c>
       <x:c r="G3" s="14" t="str">
         <x:v>Visualize module contribution and failure cases</x:v>
       </x:c>
-      <x:c r="H3" s="8" t="str">
+      <x:c r="H3" s="14" t="str">
         <x:v>ready</x:v>
       </x:c>
       <x:c r="I3" s="14" t="str">
@@ -1117,560 +1213,668 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="42" hidden="0" customHeight="1">
-      <x:c r="A4" s="17" t="n">
+      <x:c r="A4" s="115" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B4" s="115" t="str">
         <x:v>ablation-path</x:v>
       </x:c>
-      <x:c r="C4" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D4" s="8" t="str">
+      <x:c r="C4" s="115" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D4" s="115" t="str">
         <x:v>3d</x:v>
       </x:c>
-      <x:c r="E4" s="14" t="str">
+      <x:c r="E4" s="116" t="str">
         <x:v>ablation_scene2_representative_3d.png</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
+      <x:c r="F4" s="116" t="str">
         <x:v>supplement</x:v>
       </x:c>
-      <x:c r="G4" s="14" t="str">
+      <x:c r="G4" s="116" t="str">
         <x:v>Visualize module contribution and failure cases</x:v>
       </x:c>
-      <x:c r="H4" s="8" t="str">
+      <x:c r="H4" s="116" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I4" s="14" t="str">
+      <x:c r="I4" s="116" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\ablation\ablation_scene2_representative_3d.png</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" hidden="0" customHeight="1">
-      <x:c r="A5" s="63" t="n">
+      <x:c r="A5" s="119" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B5" s="55" t="str">
+      <x:c r="B5" s="119" t="str">
         <x:v>ablation-path</x:v>
       </x:c>
-      <x:c r="C5" s="63" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D5" s="55" t="str">
+      <x:c r="C5" s="119" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D5" s="119" t="str">
         <x:v>top</x:v>
       </x:c>
-      <x:c r="E5" s="64" t="str">
+      <x:c r="E5" s="120" t="str">
         <x:v>ablation_scene2_representative_top.png</x:v>
       </x:c>
-      <x:c r="F5" s="55" t="str">
+      <x:c r="F5" s="120" t="str">
         <x:v>main-text</x:v>
       </x:c>
-      <x:c r="G5" s="64" t="str">
+      <x:c r="G5" s="120" t="str">
         <x:v>Visualize module contribution and failure cases</x:v>
       </x:c>
-      <x:c r="H5" s="55" t="str">
+      <x:c r="H5" s="120" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I5" s="64" t="str">
+      <x:c r="I5" s="120" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\ablation\ablation_scene2_representative_top.png</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" hidden="0" customHeight="1">
-      <x:c r="A6" s="17" t="n">
+      <x:c r="A6" s="115" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="8" t="str">
+      <x:c r="B6" s="115" t="str">
         <x:v>ablation-path</x:v>
       </x:c>
-      <x:c r="C6" s="17" t="n">
+      <x:c r="C6" s="115" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D6" s="8" t="str">
+      <x:c r="D6" s="115" t="str">
         <x:v>3d</x:v>
       </x:c>
-      <x:c r="E6" s="14" t="str">
+      <x:c r="E6" s="116" t="str">
         <x:v>ablation_scene4_representative_3d.png</x:v>
       </x:c>
-      <x:c r="F6" s="8" t="str">
+      <x:c r="F6" s="116" t="str">
         <x:v>supplement</x:v>
       </x:c>
-      <x:c r="G6" s="14" t="str">
+      <x:c r="G6" s="116" t="str">
         <x:v>Visualize module contribution and failure cases</x:v>
       </x:c>
-      <x:c r="H6" s="8" t="str">
+      <x:c r="H6" s="116" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I6" s="14" t="str">
+      <x:c r="I6" s="116" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\ablation\ablation_scene4_representative_3d.png</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" hidden="0" customHeight="1">
-      <x:c r="A7" s="63" t="n">
+      <x:c r="A7" s="119" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B7" s="55" t="str">
+      <x:c r="B7" s="119" t="str">
         <x:v>ablation-path</x:v>
       </x:c>
-      <x:c r="C7" s="63" t="n">
+      <x:c r="C7" s="119" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D7" s="55" t="str">
+      <x:c r="D7" s="119" t="str">
         <x:v>top</x:v>
       </x:c>
-      <x:c r="E7" s="64" t="str">
+      <x:c r="E7" s="120" t="str">
         <x:v>ablation_scene4_representative_top.png</x:v>
       </x:c>
-      <x:c r="F7" s="55" t="str">
+      <x:c r="F7" s="120" t="str">
         <x:v>main-text</x:v>
       </x:c>
-      <x:c r="G7" s="64" t="str">
+      <x:c r="G7" s="120" t="str">
         <x:v>Visualize module contribution and failure cases</x:v>
       </x:c>
-      <x:c r="H7" s="55" t="str">
+      <x:c r="H7" s="120" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I7" s="64" t="str">
+      <x:c r="I7" s="120" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\ablation\ablation_scene4_representative_top.png</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" hidden="0" customHeight="1">
-      <x:c r="A8" s="63" t="n">
+      <x:c r="A8" s="115" t="str">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="55" t="str">
+      <x:c r="B8" s="115" t="str">
+        <x:v>boxplot</x:v>
+      </x:c>
+      <x:c r="C8" s="115" t="str"/>
+      <x:c r="D8" s="115" t="str">
+        <x:v>all-log</x:v>
+      </x:c>
+      <x:c r="E8" s="116" t="str">
+        <x:v>cvf_ae_boxplots_all_algorithms_log.png</x:v>
+      </x:c>
+      <x:c r="F8" s="116" t="str">
+        <x:v>supplement</x:v>
+      </x:c>
+      <x:c r="G8" s="116" t="str">
+        <x:v>Compare run distributions of all eleven algorithms</x:v>
+      </x:c>
+      <x:c r="H8" s="116" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="I8" s="116" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_paper_completion_figures_20260624_from_formal_results\cvf_ae_boxplots_all_algorithms_log.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" hidden="0" customHeight="1">
+      <x:c r="A9" s="119" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="119" t="str">
+        <x:v>boxplot</x:v>
+      </x:c>
+      <x:c r="C9" s="119" t="str"/>
+      <x:c r="D9" s="119" t="str">
+        <x:v>strong-linear</x:v>
+      </x:c>
+      <x:c r="E9" s="120" t="str">
+        <x:v>cvf_ae_boxplots_strong_algorithms.png</x:v>
+      </x:c>
+      <x:c r="F9" s="120" t="str">
+        <x:v>main-text</x:v>
+      </x:c>
+      <x:c r="G9" s="120" t="str">
+        <x:v>Compare run distributions of six strong algorithms</x:v>
+      </x:c>
+      <x:c r="H9" s="120" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="I9" s="120" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_paper_completion_figures_20260624_from_formal_results\cvf_ae_boxplots_strong_algorithms.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" hidden="0" customHeight="1">
+      <x:c r="A10" s="119" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" s="119" t="str">
         <x:v>convergence</x:v>
       </x:c>
-      <x:c r="C8" s="63" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D8" s="55" t="str">
+      <x:c r="C10" s="119" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="119" t="str">
         <x:v>mean-std</x:v>
       </x:c>
-      <x:c r="E8" s="64" t="str">
+      <x:c r="E10" s="120" t="str">
         <x:v>scene1_convergence_mean_std.png</x:v>
       </x:c>
-      <x:c r="F8" s="55" t="str">
+      <x:c r="F10" s="120" t="str">
         <x:v>main-text</x:v>
       </x:c>
-      <x:c r="G8" s="64" t="str">
+      <x:c r="G10" s="120" t="str">
         <x:v>Compare feasible-aware convergence behavior</x:v>
       </x:c>
-      <x:c r="H8" s="55" t="str">
+      <x:c r="H10" s="120" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I8" s="64" t="str">
+      <x:c r="I10" s="120" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_convergence_curves_20260623_from_main_comparison\scene1_convergence_mean_std.png</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="42" hidden="0" customHeight="1">
-      <x:c r="A9" s="63" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B9" s="55" t="str">
+    <x:row r="11" ht="42" hidden="0" customHeight="1">
+      <x:c r="A11" s="119" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B11" s="119" t="str">
         <x:v>convergence</x:v>
       </x:c>
-      <x:c r="C9" s="63" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D9" s="55" t="str">
+      <x:c r="C11" s="119" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D11" s="119" t="str">
         <x:v>mean-std</x:v>
       </x:c>
-      <x:c r="E9" s="64" t="str">
+      <x:c r="E11" s="120" t="str">
         <x:v>scene2_convergence_mean_std.png</x:v>
       </x:c>
-      <x:c r="F9" s="55" t="str">
+      <x:c r="F11" s="120" t="str">
         <x:v>main-text</x:v>
       </x:c>
-      <x:c r="G9" s="64" t="str">
+      <x:c r="G11" s="120" t="str">
         <x:v>Compare feasible-aware convergence behavior</x:v>
       </x:c>
-      <x:c r="H9" s="55" t="str">
+      <x:c r="H11" s="120" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I9" s="64" t="str">
+      <x:c r="I11" s="120" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_convergence_curves_20260623_from_main_comparison\scene2_convergence_mean_std.png</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="42" hidden="0" customHeight="1">
-      <x:c r="A10" s="63" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B10" s="55" t="str">
+    <x:row r="12" ht="42" hidden="0" customHeight="1">
+      <x:c r="A12" s="119" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B12" s="119" t="str">
         <x:v>convergence</x:v>
       </x:c>
-      <x:c r="C10" s="63" t="n">
+      <x:c r="C12" s="119" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D10" s="55" t="str">
+      <x:c r="D12" s="119" t="str">
         <x:v>mean-std</x:v>
       </x:c>
-      <x:c r="E10" s="64" t="str">
+      <x:c r="E12" s="120" t="str">
         <x:v>scene4_convergence_mean_std.png</x:v>
       </x:c>
-      <x:c r="F10" s="55" t="str">
+      <x:c r="F12" s="120" t="str">
         <x:v>main-text</x:v>
       </x:c>
-      <x:c r="G10" s="64" t="str">
+      <x:c r="G12" s="120" t="str">
         <x:v>Compare feasible-aware convergence behavior</x:v>
       </x:c>
-      <x:c r="H10" s="55" t="str">
+      <x:c r="H12" s="120" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I10" s="64" t="str">
+      <x:c r="I12" s="120" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_convergence_curves_20260623_from_main_comparison\scene4_convergence_mean_std.png</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="42" hidden="0" customHeight="1">
-      <x:c r="A11" s="17" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B11" s="8" t="str">
-        <x:v>extended-path</x:v>
-      </x:c>
-      <x:c r="C11" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D11" s="8" t="str">
-        <x:v>3d</x:v>
-      </x:c>
-      <x:c r="E11" s="14" t="str">
-        <x:v>extended_scene1_representative_3d.png</x:v>
-      </x:c>
-      <x:c r="F11" s="8" t="str">
-        <x:v>supplement</x:v>
-      </x:c>
-      <x:c r="G11" s="14" t="str">
-        <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
-      </x:c>
-      <x:c r="H11" s="8" t="str">
-        <x:v>ready</x:v>
-      </x:c>
-      <x:c r="I11" s="14" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene1_representative_3d.png</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="42" hidden="0" customHeight="1">
-      <x:c r="A12" s="63" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B12" s="55" t="str">
-        <x:v>extended-path</x:v>
-      </x:c>
-      <x:c r="C12" s="63" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D12" s="55" t="str">
-        <x:v>top</x:v>
-      </x:c>
-      <x:c r="E12" s="64" t="str">
-        <x:v>extended_scene1_representative_top.png</x:v>
-      </x:c>
-      <x:c r="F12" s="55" t="str">
-        <x:v>main-text</x:v>
-      </x:c>
-      <x:c r="G12" s="64" t="str">
-        <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
-      </x:c>
-      <x:c r="H12" s="55" t="str">
-        <x:v>ready</x:v>
-      </x:c>
-      <x:c r="I12" s="64" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene1_representative_top.png</x:v>
-      </x:c>
-    </x:row>
     <x:row r="13" ht="42" hidden="0" customHeight="1">
-      <x:c r="A13" s="17" t="n">
+      <x:c r="A13" s="8" t="str">
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="8" t="str">
         <x:v>extended-path</x:v>
       </x:c>
-      <x:c r="C13" s="17" t="n">
-        <x:v>2</x:v>
+      <x:c r="C13" s="8" t="str">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="8" t="str">
         <x:v>3d</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>extended_scene2_representative_3d.png</x:v>
-      </x:c>
-      <x:c r="F13" s="8" t="str">
+        <x:v>extended_scene1_representative_3d.png</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
         <x:v>supplement</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
         <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
       </x:c>
-      <x:c r="H13" s="8" t="str">
+      <x:c r="H13" s="14" t="str">
         <x:v>ready</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene2_representative_3d.png</x:v>
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene1_representative_3d.png</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" hidden="0" customHeight="1">
-      <x:c r="A14" s="63" t="n">
+      <x:c r="A14" s="119" t="str">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B14" s="55" t="str">
+      <x:c r="B14" s="119" t="str">
         <x:v>extended-path</x:v>
       </x:c>
-      <x:c r="C14" s="63" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D14" s="55" t="str">
+      <x:c r="C14" s="119" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="119" t="str">
         <x:v>top</x:v>
       </x:c>
-      <x:c r="E14" s="64" t="str">
-        <x:v>extended_scene2_representative_top.png</x:v>
-      </x:c>
-      <x:c r="F14" s="55" t="str">
+      <x:c r="E14" s="120" t="str">
+        <x:v>extended_scene1_representative_top.png</x:v>
+      </x:c>
+      <x:c r="F14" s="120" t="str">
         <x:v>main-text</x:v>
       </x:c>
-      <x:c r="G14" s="64" t="str">
+      <x:c r="G14" s="120" t="str">
         <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
       </x:c>
-      <x:c r="H14" s="55" t="str">
+      <x:c r="H14" s="120" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I14" s="64" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene2_representative_top.png</x:v>
+      <x:c r="I14" s="120" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene1_representative_top.png</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" hidden="0" customHeight="1">
-      <x:c r="A15" s="17" t="n">
+      <x:c r="A15" s="8" t="str">
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="8" t="str">
         <x:v>extended-path</x:v>
       </x:c>
-      <x:c r="C15" s="17" t="n">
-        <x:v>4</x:v>
+      <x:c r="C15" s="8" t="str">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D15" s="8" t="str">
         <x:v>3d</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>extended_scene4_representative_3d.png</x:v>
-      </x:c>
-      <x:c r="F15" s="8" t="str">
+        <x:v>extended_scene2_representative_3d.png</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
         <x:v>supplement</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
         <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
       </x:c>
-      <x:c r="H15" s="8" t="str">
+      <x:c r="H15" s="14" t="str">
         <x:v>ready</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene4_representative_3d.png</x:v>
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene2_representative_3d.png</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" hidden="0" customHeight="1">
-      <x:c r="A16" s="63" t="n">
+      <x:c r="A16" s="119" t="str">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B16" s="55" t="str">
+      <x:c r="B16" s="119" t="str">
         <x:v>extended-path</x:v>
       </x:c>
-      <x:c r="C16" s="63" t="n">
+      <x:c r="C16" s="119" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D16" s="119" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="E16" s="120" t="str">
+        <x:v>extended_scene2_representative_top.png</x:v>
+      </x:c>
+      <x:c r="F16" s="120" t="str">
+        <x:v>main-text</x:v>
+      </x:c>
+      <x:c r="G16" s="120" t="str">
+        <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
+      </x:c>
+      <x:c r="H16" s="120" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="I16" s="120" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene2_representative_top.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" hidden="0" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>extended-path</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
         <x:v>4</x:v>
-      </x:c>
-      <x:c r="D16" s="55" t="str">
-        <x:v>top</x:v>
-      </x:c>
-      <x:c r="E16" s="64" t="str">
-        <x:v>extended_scene4_representative_top.png</x:v>
-      </x:c>
-      <x:c r="F16" s="55" t="str">
-        <x:v>main-text</x:v>
-      </x:c>
-      <x:c r="G16" s="64" t="str">
-        <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
-      </x:c>
-      <x:c r="H16" s="55" t="str">
-        <x:v>ready</x:v>
-      </x:c>
-      <x:c r="I16" s="64" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene4_representative_top.png</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="42" hidden="0" customHeight="1">
-      <x:c r="A17" s="17" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B17" s="8" t="str">
-        <x:v>main-path</x:v>
-      </x:c>
-      <x:c r="C17" s="17" t="n">
-        <x:v>1</x:v>
       </x:c>
       <x:c r="D17" s="8" t="str">
         <x:v>3d</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>main_scene1_representative_3d.png</x:v>
-      </x:c>
-      <x:c r="F17" s="8" t="str">
+        <x:v>extended_scene4_representative_3d.png</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="str">
         <x:v>supplement</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>Classic-baseline representative path comparison</x:v>
-      </x:c>
-      <x:c r="H17" s="8" t="str">
+        <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
+      </x:c>
+      <x:c r="H17" s="14" t="str">
         <x:v>ready</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene1_representative_3d.png</x:v>
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene4_representative_3d.png</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" hidden="0" customHeight="1">
-      <x:c r="A18" s="17" t="n">
+      <x:c r="A18" s="119" t="str">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B18" s="8" t="str">
-        <x:v>main-path</x:v>
-      </x:c>
-      <x:c r="C18" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D18" s="8" t="str">
+      <x:c r="B18" s="119" t="str">
+        <x:v>extended-path</x:v>
+      </x:c>
+      <x:c r="C18" s="119" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D18" s="119" t="str">
         <x:v>top</x:v>
       </x:c>
-      <x:c r="E18" s="14" t="str">
-        <x:v>main_scene1_representative_top.png</x:v>
-      </x:c>
-      <x:c r="F18" s="8" t="str">
-        <x:v>supplement</x:v>
-      </x:c>
-      <x:c r="G18" s="14" t="str">
-        <x:v>Classic-baseline representative path comparison</x:v>
-      </x:c>
-      <x:c r="H18" s="8" t="str">
+      <x:c r="E18" s="120" t="str">
+        <x:v>extended_scene4_representative_top.png</x:v>
+      </x:c>
+      <x:c r="F18" s="120" t="str">
+        <x:v>main-text</x:v>
+      </x:c>
+      <x:c r="G18" s="120" t="str">
+        <x:v>Compare CVF-AE with strong and recent improved methods</x:v>
+      </x:c>
+      <x:c r="H18" s="120" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I18" s="14" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene1_representative_top.png</x:v>
+      <x:c r="I18" s="120" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\extended\extended_scene4_representative_top.png</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" hidden="0" customHeight="1">
-      <x:c r="A19" s="17" t="n">
+      <x:c r="A19" s="8" t="str">
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="8" t="str">
         <x:v>main-path</x:v>
       </x:c>
-      <x:c r="C19" s="17" t="n">
-        <x:v>2</x:v>
+      <x:c r="C19" s="8" t="str">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D19" s="8" t="str">
         <x:v>3d</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>main_scene2_representative_3d.png</x:v>
-      </x:c>
-      <x:c r="F19" s="8" t="str">
+        <x:v>main_scene1_representative_3d.png</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
         <x:v>supplement</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
         <x:v>Classic-baseline representative path comparison</x:v>
       </x:c>
-      <x:c r="H19" s="8" t="str">
+      <x:c r="H19" s="14" t="str">
         <x:v>ready</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene2_representative_3d.png</x:v>
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene1_representative_3d.png</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" hidden="0" customHeight="1">
-      <x:c r="A20" s="17" t="n">
+      <x:c r="A20" s="115" t="str">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B20" s="8" t="str">
+      <x:c r="B20" s="115" t="str">
         <x:v>main-path</x:v>
       </x:c>
-      <x:c r="C20" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D20" s="8" t="str">
+      <x:c r="C20" s="115" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="115" t="str">
         <x:v>top</x:v>
       </x:c>
-      <x:c r="E20" s="14" t="str">
-        <x:v>main_scene2_representative_top.png</x:v>
-      </x:c>
-      <x:c r="F20" s="8" t="str">
+      <x:c r="E20" s="116" t="str">
+        <x:v>main_scene1_representative_top.png</x:v>
+      </x:c>
+      <x:c r="F20" s="116" t="str">
         <x:v>supplement</x:v>
       </x:c>
-      <x:c r="G20" s="14" t="str">
+      <x:c r="G20" s="116" t="str">
         <x:v>Classic-baseline representative path comparison</x:v>
       </x:c>
-      <x:c r="H20" s="8" t="str">
+      <x:c r="H20" s="116" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I20" s="14" t="str">
-        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene2_representative_top.png</x:v>
+      <x:c r="I20" s="116" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene1_representative_top.png</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" hidden="0" customHeight="1">
-      <x:c r="A21" s="17" t="n">
+      <x:c r="A21" s="8" t="str">
         <x:v>20</x:v>
       </x:c>
       <x:c r="B21" s="8" t="str">
         <x:v>main-path</x:v>
       </x:c>
-      <x:c r="C21" s="17" t="n">
-        <x:v>4</x:v>
+      <x:c r="C21" s="8" t="str">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D21" s="8" t="str">
         <x:v>3d</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>main_scene4_representative_3d.png</x:v>
-      </x:c>
-      <x:c r="F21" s="8" t="str">
+        <x:v>main_scene2_representative_3d.png</x:v>
+      </x:c>
+      <x:c r="F21" s="14" t="str">
         <x:v>supplement</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
         <x:v>Classic-baseline representative path comparison</x:v>
       </x:c>
-      <x:c r="H21" s="8" t="str">
+      <x:c r="H21" s="14" t="str">
         <x:v>ready</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene2_representative_3d.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="42" hidden="0" customHeight="1">
+      <x:c r="A22" s="115" t="str">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B22" s="115" t="str">
+        <x:v>main-path</x:v>
+      </x:c>
+      <x:c r="C22" s="115" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D22" s="115" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="E22" s="116" t="str">
+        <x:v>main_scene2_representative_top.png</x:v>
+      </x:c>
+      <x:c r="F22" s="116" t="str">
+        <x:v>supplement</x:v>
+      </x:c>
+      <x:c r="G22" s="116" t="str">
+        <x:v>Classic-baseline representative path comparison</x:v>
+      </x:c>
+      <x:c r="H22" s="116" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="I22" s="116" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene2_representative_top.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="8" t="str">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>main-path</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D23" s="8" t="str">
+        <x:v>3d</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="str">
+        <x:v>main_scene4_representative_3d.png</x:v>
+      </x:c>
+      <x:c r="F23" s="14" t="str">
+        <x:v>supplement</x:v>
+      </x:c>
+      <x:c r="G23" s="14" t="str">
+        <x:v>Classic-baseline representative path comparison</x:v>
+      </x:c>
+      <x:c r="H23" s="14" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="I23" s="14" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene4_representative_3d.png</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="42" hidden="0" customHeight="1">
-      <x:c r="A22" s="17" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B22" s="8" t="str">
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="115" t="str">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B24" s="115" t="str">
         <x:v>main-path</x:v>
       </x:c>
-      <x:c r="C22" s="17" t="n">
+      <x:c r="C24" s="115" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D22" s="8" t="str">
+      <x:c r="D24" s="115" t="str">
         <x:v>top</x:v>
       </x:c>
-      <x:c r="E22" s="14" t="str">
+      <x:c r="E24" s="116" t="str">
         <x:v>main_scene4_representative_top.png</x:v>
       </x:c>
-      <x:c r="F22" s="8" t="str">
+      <x:c r="F24" s="116" t="str">
         <x:v>supplement</x:v>
       </x:c>
-      <x:c r="G22" s="14" t="str">
+      <x:c r="G24" s="116" t="str">
         <x:v>Classic-baseline representative path comparison</x:v>
       </x:c>
-      <x:c r="H22" s="8" t="str">
+      <x:c r="H24" s="116" t="str">
         <x:v>ready</x:v>
       </x:c>
-      <x:c r="I22" s="14" t="str">
+      <x:c r="I24" s="116" t="str">
         <x:v>routes\route_b_cvf_ae\results\cvf_ae_representative_paths_20260623_from_formal_results\main\main_scene4_representative_top.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="119" t="str">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" s="119" t="str">
+        <x:v>method</x:v>
+      </x:c>
+      <x:c r="C25" s="119" t="str"/>
+      <x:c r="D25" s="119" t="str">
+        <x:v>flowchart</x:v>
+      </x:c>
+      <x:c r="E25" s="120" t="str">
+        <x:v>cvf_ae_method_flowchart.png</x:v>
+      </x:c>
+      <x:c r="F25" s="120" t="str">
+        <x:v>main-text</x:v>
+      </x:c>
+      <x:c r="G25" s="120" t="str">
+        <x:v>Present the complete CVF-AE procedure</x:v>
+      </x:c>
+      <x:c r="H25" s="120" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="I25" s="120" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_paper_completion_figures_20260624_from_formal_results\cvf_ae_method_flowchart.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="119" t="str">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" s="119" t="str">
+        <x:v>parameter-sensitivity</x:v>
+      </x:c>
+      <x:c r="C26" s="119" t="str"/>
+      <x:c r="D26" s="119" t="str">
+        <x:v>mean-std</x:v>
+      </x:c>
+      <x:c r="E26" s="120" t="str">
+        <x:v>cvf_ae_parameter_sensitivity.png</x:v>
+      </x:c>
+      <x:c r="F26" s="120" t="str">
+        <x:v>main-text</x:v>
+      </x:c>
+      <x:c r="G26" s="120" t="str">
+        <x:v>Evaluate robustness to key CVF parameters</x:v>
+      </x:c>
+      <x:c r="H26" s="120" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="I26" s="120" t="str">
+        <x:v>routes\route_b_cvf_ae\results\cvf_ae_paper_completion_figures_20260624_from_formal_results\cvf_ae_parameter_sensitivity.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd27ef4b8957b4d07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e1e429ea0a46d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2152,7 +2356,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R324a32778e5549c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa19dae785f34bd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3822,7 +4026,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd42d90721b004a3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a7083109098478d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5026,7 +5230,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff0b057ed5934b0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf715fa9ccb824558"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5878,7 +6082,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a9e584f45f549fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R134d3259c7094814"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6512,7 +6716,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R437b8fc378e5467f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf89cfcf65e0a4904"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7376,7 +7580,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdf05d14336e4226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5512fea505c47fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8810,7 +9014,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26279432754046c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d96c7e129434459"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10128,7 +10332,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfbf8bce00e14295"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c1ce9f32408407b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>